<commit_message>
Defined testcase class in test_bank_account.py to test BankAccount, defined setUp as well as test class for __init__ for BankAccount class.
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_bank_account.xlsx
+++ b/tests/A01_pixell_test_plan_bank_account.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lauri\Desktop\Intermediate Software Development0315\2. Assignments\updated_again_0416\assignment_01\starter (given)\tests\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment_01/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE671229-BC9B-45DF-8946-EDA774314A88}"/>
   <bookViews>
-    <workbookView xWindow="31140" yWindow="2340" windowWidth="25185" windowHeight="13845" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="70">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -282,6 +282,117 @@
   </si>
   <si>
     <t>returns client number attribute</t>
+  </si>
+  <si>
+    <t>BankAccount(404, 123, 93000)</t>
+  </si>
+  <si>
+    <t>account_number = 404</t>
+  </si>
+  <si>
+    <t>account_number = 404               client_number = 123                         balance = 93000</t>
+  </si>
+  <si>
+    <t>balance = "93000"</t>
+  </si>
+  <si>
+    <t>BankAccount(404, 123, "93000")</t>
+  </si>
+  <si>
+    <t>BankAccount("404", 123, 93000)</t>
+  </si>
+  <si>
+    <t>account_number = "404"</t>
+  </si>
+  <si>
+    <t>ValueError(Balance is not of a float type.)</t>
+  </si>
+  <si>
+    <t>ValueError(Account Number must be of a numeric type.)</t>
+  </si>
+  <si>
+    <t>BankAccount(404, "123", 93000)</t>
+  </si>
+  <si>
+    <t>client_number = "123"</t>
+  </si>
+  <si>
+    <t>ValueError(Client Number must be of a numeric type.)</t>
+  </si>
+  <si>
+    <t>client_number = 123</t>
+  </si>
+  <si>
+    <t>balance = 93000</t>
+  </si>
+  <si>
+    <t>BankAccount.update_balance(1000)</t>
+  </si>
+  <si>
+    <t>BankAccount.update_balance(-1000)</t>
+  </si>
+  <si>
+    <t>BankAccount.update_balance("1000")</t>
+  </si>
+  <si>
+    <t>BankAccount.deposit(1000)</t>
+  </si>
+  <si>
+    <t>BankAccount.deposit(-1000)</t>
+  </si>
+  <si>
+    <t>BankAccount.withdraw(1000)</t>
+  </si>
+  <si>
+    <t>BankAccount.withdraw(-1000)</t>
+  </si>
+  <si>
+    <t>BankAccount.withdraw(94000)</t>
+  </si>
+  <si>
+    <t>.update_balance(1000)</t>
+  </si>
+  <si>
+    <t>balance = 94000</t>
+  </si>
+  <si>
+    <t>.update_balance(-1000)</t>
+  </si>
+  <si>
+    <t>balance = 92000</t>
+  </si>
+  <si>
+    <t>.update_balance("1000")</t>
+  </si>
+  <si>
+    <t>ValueError(Amount must be of a numeric type.)</t>
+  </si>
+  <si>
+    <t>.deposit(1000)</t>
+  </si>
+  <si>
+    <t>.deposit(-1000)</t>
+  </si>
+  <si>
+    <t>ValueError(Deposit amount:   -1000 must be positive.)</t>
+  </si>
+  <si>
+    <t>.withdraw(1000)</t>
+  </si>
+  <si>
+    <t>.withdraw(-1000)</t>
+  </si>
+  <si>
+    <t>.withdraw(94000)</t>
+  </si>
+  <si>
+    <t>ValueError(Withdraw amount: 94000 must not exceed the account balance: 93000)</t>
+  </si>
+  <si>
+    <t>print(BankAccount)</t>
+  </si>
+  <si>
+    <t>Account Number: 404 Balance: $93,000.00</t>
   </si>
 </sst>
 </file>
@@ -619,6 +730,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -642,12 +759,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1207,29 +1318,29 @@
       <c r="B2" s="2" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="19"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="19"/>
+      <c r="D4" s="21"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
@@ -1258,15 +1369,21 @@
       <c r="B7" s="10">
         <v>1</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="E7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="8" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1278,23 +1395,35 @@
       <c r="D8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
+      <c r="E8" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="13">
         <v>3</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
+      <c r="E9" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="10">
@@ -1306,23 +1435,35 @@
       <c r="D10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="E10" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="10">
         <v>5</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="E11" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="12" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="10">
@@ -1334,23 +1475,35 @@
       <c r="D12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+      <c r="E12" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="13" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
         <v>7</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
+      <c r="E13" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="14" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="13">
@@ -1362,23 +1515,35 @@
       <c r="D14" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
+      <c r="E14" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="15" spans="2:7" ht="47.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="10">
         <v>9</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="E15" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="16" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="10">
@@ -1390,23 +1555,35 @@
       <c r="D16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="E16" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="17" spans="2:7" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="10">
         <v>11</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
+      <c r="E17" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="18" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="3">
@@ -1418,23 +1595,35 @@
       <c r="D18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="E18" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="19" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="13">
         <v>13</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="E19" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="20" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="10">
@@ -1446,23 +1635,35 @@
       <c r="D20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="E20" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="21" spans="2:7" ht="31.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="10">
         <v>15</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
+      <c r="E21" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10">
@@ -1474,9 +1675,15 @@
       <c r="D22" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="E22" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="23" spans="2:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="3">
@@ -1629,14 +1836,14 @@
       <c r="G37" s="5"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="21"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
+      <c r="G39" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Completed pre unit teseting spreadsheet as well as defined all unit tests for BanckAccount class, all working properly, also adjusted code to resolve testing issue and correct mistakes.
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_bank_account.xlsx
+++ b/tests/A01_pixell_test_plan_bank_account.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment_01/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE671229-BC9B-45DF-8946-EDA774314A88}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F542F5C1-D348-423F-892A-B8C40F915818}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-16320" yWindow="-4530" windowWidth="16440" windowHeight="28320" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="71">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -393,6 +393,9 @@
   </si>
   <si>
     <t>Account Number: 404 Balance: $93,000.00</t>
+  </si>
+  <si>
+    <t>Trevor Donald</t>
   </si>
 </sst>
 </file>
@@ -905,6 +908,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1330,7 +1337,9 @@
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="18"/>
+      <c r="C3" s="18" t="s">
+        <v>70</v>
+      </c>
       <c r="D3" s="19"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added unittesting for ChquingAccount and ensured everything functions properly
</commit_message>
<xml_diff>
--- a/tests/A01_pixell_test_plan_bank_account.xlsx
+++ b/tests/A01_pixell_test_plan_bank_account.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment_01/tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{56DA4A4F-2E79-4753-B9BE-A428E4C99413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F542F5C1-D348-423F-892A-B8C40F915818}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-4530" windowWidth="16440" windowHeight="28320" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="25695" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -908,10 +908,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>